<commit_message>
updated codebook in spreadsheet format
</commit_message>
<xml_diff>
--- a/institutionaldata/HHMI_IE3_codebook.xlsx
+++ b/institutionaldata/HHMI_IE3_codebook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Research\Research Projects\GSU\HHMI_IE3\Analyses\HHMI_Student_Success\institutionaldata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EB2E684-6206-47A0-B2C6-E3C4A2D978FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97A04B24-4F1C-4D2F-85FF-B2A6374F616B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-2085" yWindow="-21360" windowWidth="30330" windowHeight="21225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25485" yWindow="0" windowWidth="25815" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="codebook" sheetId="1" r:id="rId1"/>
@@ -56,9 +56,6 @@
     <t>student_ID</t>
   </si>
   <si>
-    <t>WHKEY,ID,PantherID,SDSTUMAIN_WHKEY,Student_ID,Pidm</t>
-  </si>
-  <si>
     <t>flag_first_generation</t>
   </si>
   <si>
@@ -694,6 +691,9 @@
   </si>
   <si>
     <t>WHKEY_INSTRUCTOR</t>
+  </si>
+  <si>
+    <t>WHKEY,ID,PantherID,SDSTUDEMOG_WHKEY,SDSTUMAIN_WHKEY,Student_ID,Pidm</t>
   </si>
 </sst>
 </file>
@@ -1589,14 +1589,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F39"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="54.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="93.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="54.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="93.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1607,483 +1607,483 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
       </c>
       <c r="F1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" t="s">
         <v>63</v>
       </c>
-      <c r="B2" t="s">
-        <v>64</v>
-      </c>
       <c r="D2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" t="s">
         <v>65</v>
       </c>
-      <c r="B3" t="s">
-        <v>66</v>
-      </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" t="s">
         <v>61</v>
       </c>
-      <c r="B4" t="s">
-        <v>62</v>
-      </c>
       <c r="D4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" t="s">
         <v>67</v>
       </c>
-      <c r="B5" t="s">
-        <v>68</v>
-      </c>
       <c r="C5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
         <v>19</v>
       </c>
-      <c r="B6" t="s">
-        <v>20</v>
-      </c>
       <c r="C6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
         <v>21</v>
       </c>
-      <c r="B7" t="s">
-        <v>22</v>
-      </c>
       <c r="C7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" t="s">
         <v>35</v>
       </c>
-      <c r="B8" t="s">
-        <v>36</v>
-      </c>
       <c r="C8" t="s">
+        <v>81</v>
+      </c>
+      <c r="D8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" t="s">
         <v>82</v>
-      </c>
-      <c r="D8" t="s">
-        <v>80</v>
-      </c>
-      <c r="E8" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" t="s">
         <v>37</v>
       </c>
-      <c r="B9" t="s">
-        <v>38</v>
-      </c>
       <c r="C9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D9" t="s">
+        <v>79</v>
+      </c>
+      <c r="E9" t="s">
         <v>85</v>
       </c>
-      <c r="D9" t="s">
-        <v>80</v>
-      </c>
-      <c r="E9" t="s">
-        <v>86</v>
-      </c>
       <c r="F9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
+        <v>131</v>
+      </c>
+      <c r="D10" t="s">
         <v>132</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>133</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>134</v>
-      </c>
-      <c r="F10" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s">
         <v>23</v>
       </c>
-      <c r="B11" t="s">
-        <v>24</v>
-      </c>
       <c r="C11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D11" t="s">
+        <v>79</v>
+      </c>
+      <c r="E11" t="s">
         <v>87</v>
-      </c>
-      <c r="D11" t="s">
-        <v>80</v>
-      </c>
-      <c r="E11" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
+        <v>137</v>
+      </c>
+      <c r="B12" t="s">
         <v>138</v>
-      </c>
-      <c r="B12" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" t="s">
         <v>27</v>
       </c>
-      <c r="B13" t="s">
-        <v>28</v>
-      </c>
       <c r="C13" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" t="s">
         <v>25</v>
       </c>
-      <c r="B14" t="s">
-        <v>26</v>
-      </c>
       <c r="C14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" t="s">
         <v>29</v>
       </c>
-      <c r="B15" t="s">
-        <v>30</v>
-      </c>
       <c r="C15" t="s">
+        <v>90</v>
+      </c>
+      <c r="D15" t="s">
+        <v>79</v>
+      </c>
+      <c r="E15" t="s">
         <v>91</v>
-      </c>
-      <c r="D15" t="s">
-        <v>80</v>
-      </c>
-      <c r="E15" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" t="s">
         <v>31</v>
       </c>
-      <c r="B16" t="s">
-        <v>32</v>
-      </c>
       <c r="C16" t="s">
+        <v>92</v>
+      </c>
+      <c r="D16" t="s">
+        <v>80</v>
+      </c>
+      <c r="E16" t="s">
         <v>93</v>
-      </c>
-      <c r="D16" t="s">
-        <v>81</v>
-      </c>
-      <c r="E16" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
         <v>33</v>
       </c>
-      <c r="B17" t="s">
-        <v>34</v>
-      </c>
       <c r="C17" t="s">
+        <v>94</v>
+      </c>
+      <c r="D17" t="s">
         <v>95</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>96</v>
-      </c>
-      <c r="E17" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" t="s">
         <v>55</v>
       </c>
-      <c r="B18" t="s">
-        <v>56</v>
-      </c>
       <c r="C18" t="s">
+        <v>97</v>
+      </c>
+      <c r="D18" t="s">
+        <v>80</v>
+      </c>
+      <c r="E18" t="s">
         <v>98</v>
-      </c>
-      <c r="D18" t="s">
-        <v>81</v>
-      </c>
-      <c r="E18" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C19" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" t="s">
         <v>47</v>
       </c>
-      <c r="B20" t="s">
-        <v>48</v>
-      </c>
       <c r="C20" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E20" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" t="s">
         <v>43</v>
       </c>
-      <c r="B21" t="s">
-        <v>44</v>
-      </c>
       <c r="D21" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F21" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" t="s">
         <v>45</v>
       </c>
-      <c r="B22" t="s">
-        <v>46</v>
-      </c>
       <c r="D22" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
+        <v>48</v>
+      </c>
+      <c r="B23" t="s">
         <v>49</v>
-      </c>
-      <c r="B23" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" t="s">
         <v>51</v>
-      </c>
-      <c r="B24" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" t="s">
         <v>53</v>
       </c>
-      <c r="B25" t="s">
-        <v>54</v>
-      </c>
       <c r="C25" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D25" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E25" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
+        <v>11</v>
+      </c>
+      <c r="B26" t="s">
         <v>12</v>
       </c>
-      <c r="B26" t="s">
-        <v>13</v>
-      </c>
       <c r="C26" t="s">
+        <v>100</v>
+      </c>
+      <c r="D26" t="s">
+        <v>99</v>
+      </c>
+      <c r="E26" t="s">
         <v>101</v>
       </c>
-      <c r="D26" t="s">
-        <v>100</v>
-      </c>
-      <c r="E26" t="s">
-        <v>102</v>
-      </c>
       <c r="F26" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C27" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D27" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E27" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F27" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C28" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D28" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E28" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F28" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" t="s">
+        <v>15</v>
+      </c>
+      <c r="B29" t="s">
         <v>16</v>
       </c>
-      <c r="B29" t="s">
-        <v>17</v>
-      </c>
       <c r="C29" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D29" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E29" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F29" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C30" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E30" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F30" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" t="s">
         <v>58</v>
-      </c>
-      <c r="B31" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C32" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D32" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E32" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -2091,13 +2091,13 @@
         <v>7</v>
       </c>
       <c r="C33" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D33" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -2108,13 +2108,13 @@
         <v>4</v>
       </c>
       <c r="C34" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D34" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E34" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -2125,13 +2125,13 @@
         <v>6</v>
       </c>
       <c r="C35" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D35" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E35" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -2139,33 +2139,33 @@
         <v>10</v>
       </c>
       <c r="B36" t="s">
-        <v>11</v>
+        <v>139</v>
       </c>
       <c r="C36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D36" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E36" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B37" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C37" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D37" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -2176,30 +2176,30 @@
         <v>9</v>
       </c>
       <c r="C38" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D38" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E38" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
+        <v>39</v>
+      </c>
+      <c r="B39" t="s">
         <v>40</v>
       </c>
-      <c r="B39" t="s">
-        <v>41</v>
-      </c>
       <c r="C39" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D39" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E39" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -2213,36 +2213,36 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
addition of a couple helper functions; general code cleanup
</commit_message>
<xml_diff>
--- a/institutionaldata/HHMI_IE3_codebook.xlsx
+++ b/institutionaldata/HHMI_IE3_codebook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Research\Research Projects\GSU\HHMI_IE3\Analyses\HHMI_Student_Success\institutionaldata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A09C1CD-4D62-479D-B5C4-34B85E09FBDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B358AD3-DFE8-4FA6-955B-F5AC9BCA762B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25485" yWindow="0" windowWidth="25815" windowHeight="20625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24210" yWindow="-21600" windowWidth="25800" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="codebook" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="191">
   <si>
     <t>variable_name_project</t>
   </si>
@@ -556,7 +556,284 @@
   </si>
   <si>
     <r>
-      <t>degree program, abbreviated (</t>
+      <t>major, abbreviated (</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">e.g. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BIO)</t>
+    </r>
+  </si>
+  <si>
+    <t>transfer credits associated with current term</t>
+  </si>
+  <si>
+    <t># This file is used by utilityfunctions.rename_columns_in_bulk() in order to rename columns to a standardized format</t>
+  </si>
+  <si>
+    <t># for multi-institutional usage. variable_name_project is a column comprised in which standard field names are placed,</t>
+  </si>
+  <si>
+    <t># and variable_name_institution holds comma-separated variants that refer to this variable at any institution. Do not</t>
+  </si>
+  <si>
+    <t># include any white spaces after the comma in the list.</t>
+  </si>
+  <si>
+    <t># The description column is provided so we can write out common definitions</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t># column_mapping.xlsx</t>
+  </si>
+  <si>
+    <t>Character</t>
+  </si>
+  <si>
+    <t>Y or N</t>
+  </si>
+  <si>
+    <t>Can be derived from function?</t>
+  </si>
+  <si>
+    <t>utilityfunctions.letter_grade_simplify()</t>
+  </si>
+  <si>
+    <t>student ID number; ciphering with utilityfunctions.scramble_ID() is advised</t>
+  </si>
+  <si>
+    <t>utilityfunctions.set_up_demographic_flags()</t>
+  </si>
+  <si>
+    <t>high school CEEB (College Entrance Examination Board) code</t>
+  </si>
+  <si>
+    <t>typically 6 digits (with exceptions for international schools)</t>
+  </si>
+  <si>
+    <t>*normalization can be performed via utilityfunctions.num_grade_normalized()</t>
+  </si>
+  <si>
+    <t>course_grade_numeric</t>
+  </si>
+  <si>
+    <t>Float</t>
+  </si>
+  <si>
+    <t>numeric equivalent to letter grade</t>
+  </si>
+  <si>
+    <t>utilityfunctions.num_grade_institutional() and normalization with utilityfunctions.num_grade_normalized()</t>
+  </si>
+  <si>
+    <t>represents year and month of term for demographics</t>
+  </si>
+  <si>
+    <t>varies by institution</t>
+  </si>
+  <si>
+    <t>course_instructor_id</t>
+  </si>
+  <si>
+    <t>WHKEY_INSTRUCTOR</t>
+  </si>
+  <si>
+    <t>WHKEY,ID,PantherID,SDSTUDEMOG_WHKEY,SDSTUMAIN_WHKEY,Student_ID,Pidm</t>
+  </si>
+  <si>
+    <t>Grad_date, GRAD_DATE</t>
+  </si>
+  <si>
+    <t>Date Time</t>
+  </si>
+  <si>
+    <t>represents year and month of matriculation term (WARNING: AT GSU THIS IS UNRELIABLE)</t>
+  </si>
+  <si>
+    <t>matriculation_term</t>
+  </si>
+  <si>
+    <t>graduation_status</t>
+  </si>
+  <si>
+    <t>Awarded, Pending, etc</t>
+  </si>
+  <si>
+    <t>demographics_age_term</t>
+  </si>
+  <si>
+    <t>AGE_TERM</t>
+  </si>
+  <si>
+    <t>term_earliest</t>
+  </si>
+  <si>
+    <t>EARLIEST_TERM</t>
+  </si>
+  <si>
+    <t>transfer_hours_term</t>
+  </si>
+  <si>
+    <t>transfer_hours_earliest_term</t>
+  </si>
+  <si>
+    <t>major_earliest_term</t>
+  </si>
+  <si>
+    <t>MAJOR_EARLIEST_TERM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRADUATION_STATUS_DESCR, </t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>flag_transfer_credits_over_11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 or 0 </t>
+  </si>
+  <si>
+    <t>indicates if a student transferred with 12+ credit hours</t>
+  </si>
+  <si>
+    <t>flag_first_attempt</t>
+  </si>
+  <si>
+    <t>indicates if student record for course represents first attempt</t>
+  </si>
+  <si>
+    <t>years_before_course</t>
+  </si>
+  <si>
+    <t>demographics_high_school_GPA_standardized</t>
+  </si>
+  <si>
+    <t>difference in years from course_term and term_earliest</t>
+  </si>
+  <si>
+    <t>(demographics_high_school_GPA - demographics_high_school_GPA for cohort starting the same entry term) / demographics_high_school_GPA for cohort starting the same entry term</t>
+  </si>
+  <si>
+    <t>discipline_earliest_term</t>
+  </si>
+  <si>
+    <t>discipline_third_year_fall</t>
+  </si>
+  <si>
+    <t>bio_sci, phy_sci, eng_cs, other_STEM, non_STEM</t>
+  </si>
+  <si>
+    <t>flag_hispanic</t>
+  </si>
+  <si>
+    <t>HISPANIC</t>
+  </si>
+  <si>
+    <t>1 = Hispanic; 0 = non-Hispanic or not reported</t>
+  </si>
+  <si>
+    <t>demographics_hispanic</t>
+  </si>
+  <si>
+    <t>1 = Hispanic; 0 = non-Hispanic, -1 = ethnicity not reported</t>
+  </si>
+  <si>
+    <t>demographics_ethnicity</t>
+  </si>
+  <si>
+    <t>ETHNICITY_CODE</t>
+  </si>
+  <si>
+    <t>2 = Hispanic; 1 = not Hispanic; nan = not reported</t>
+  </si>
+  <si>
+    <t>major,SDSTUMAIN_MAJOR,StuMajr_Code1,MAJOR_COURSETERM,MAJOR</t>
+  </si>
+  <si>
+    <t>term_earliest_us</t>
+  </si>
+  <si>
+    <t>FIRST_TERM_US_NO_RESTRICTION</t>
+  </si>
+  <si>
+    <t>represents year and month of matriculation term or start of degree (your IR data may vary in this)</t>
+  </si>
+  <si>
+    <t>represents year and month of matriculation term or start of bachelor's degree (your IR data may vary in this; at GSU, bachelors level code is US)</t>
+  </si>
+  <si>
+    <t>MAJOR_GRD, MAJOR_GRADUATED</t>
+  </si>
+  <si>
+    <t>major2_term</t>
+  </si>
+  <si>
+    <t>MAJOR2</t>
+  </si>
+  <si>
+    <r>
+      <t>second major, abbreviated (</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">e.g. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BIO)</t>
+    </r>
+  </si>
+  <si>
+    <t>second major of student associated with a specific term</t>
+  </si>
+  <si>
+    <t>term_level</t>
+  </si>
+  <si>
+    <t>DEGREE_LEVEL_ENROLLED</t>
+  </si>
+  <si>
+    <t>level of the student's degree program (associates, bachelors, etc) at term</t>
+  </si>
+  <si>
+    <t>graduation_level</t>
+  </si>
+  <si>
+    <r>
+      <t>level student is at in their degree program, abbreviated (</t>
     </r>
     <r>
       <rPr>
@@ -581,201 +858,31 @@
     </r>
   </si>
   <si>
-    <r>
-      <t>major, abbreviated (</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">e.g. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>BIO)</t>
-    </r>
-  </si>
-  <si>
-    <t>transfer credits associated with current term</t>
-  </si>
-  <si>
-    <t># This file is used by utilityfunctions.rename_columns_in_bulk() in order to rename columns to a standardized format</t>
-  </si>
-  <si>
-    <t># for multi-institutional usage. variable_name_project is a column comprised in which standard field names are placed,</t>
-  </si>
-  <si>
-    <t># and variable_name_institution holds comma-separated variants that refer to this variable at any institution. Do not</t>
-  </si>
-  <si>
-    <t># include any white spaces after the comma in the list.</t>
-  </si>
-  <si>
-    <t># The description column is provided so we can write out common definitions</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t># column_mapping.xlsx</t>
-  </si>
-  <si>
-    <t>Character</t>
-  </si>
-  <si>
-    <t>Y or N</t>
-  </si>
-  <si>
-    <t>Can be derived from function?</t>
-  </si>
-  <si>
-    <t>utilityfunctions.letter_grade_simplify()</t>
-  </si>
-  <si>
-    <t>student ID number; ciphering with utilityfunctions.scramble_ID() is advised</t>
-  </si>
-  <si>
-    <t>utilityfunctions.set_up_demographic_flags()</t>
-  </si>
-  <si>
-    <t>high school CEEB (College Entrance Examination Board) code</t>
-  </si>
-  <si>
-    <t>typically 6 digits (with exceptions for international schools)</t>
-  </si>
-  <si>
-    <t>*normalization can be performed via utilityfunctions.num_grade_normalized()</t>
-  </si>
-  <si>
-    <t>course_grade_numeric</t>
-  </si>
-  <si>
-    <t>Float</t>
-  </si>
-  <si>
-    <t>numeric equivalent to letter grade</t>
-  </si>
-  <si>
-    <t>utilityfunctions.num_grade_institutional() and normalization with utilityfunctions.num_grade_normalized()</t>
-  </si>
-  <si>
-    <t>represents year and month of term for demographics</t>
-  </si>
-  <si>
-    <t>varies by institution</t>
-  </si>
-  <si>
-    <t>course_instructor_id</t>
-  </si>
-  <si>
-    <t>WHKEY_INSTRUCTOR</t>
-  </si>
-  <si>
-    <t>WHKEY,ID,PantherID,SDSTUDEMOG_WHKEY,SDSTUMAIN_WHKEY,Student_ID,Pidm</t>
-  </si>
-  <si>
-    <t>Grad_date, GRAD_DATE</t>
-  </si>
-  <si>
-    <t>Date Time</t>
-  </si>
-  <si>
-    <t>represents year and month of matriculation term (WARNING: AT GSU THIS IS UNRELIABLE)</t>
-  </si>
-  <si>
-    <t>matriculation_term</t>
-  </si>
-  <si>
-    <t>graduation_status</t>
-  </si>
-  <si>
-    <t>Awarded, Pending, etc</t>
-  </si>
-  <si>
-    <t>demographics_age_term</t>
-  </si>
-  <si>
-    <t>AGE_TERM</t>
-  </si>
-  <si>
-    <t>term_earliest</t>
-  </si>
-  <si>
-    <t>EARLIEST_TERM</t>
-  </si>
-  <si>
-    <t>transfer_hours_term</t>
-  </si>
-  <si>
-    <t>transfer_hours_earliest_term</t>
-  </si>
-  <si>
-    <t>major_earliest_term</t>
-  </si>
-  <si>
-    <t>MAJOR_EARLIEST_TERM</t>
-  </si>
-  <si>
-    <t>major,SDSTUMAIN_MAJOR,StuMajr_Code1,MAJOR_COURSETERM</t>
-  </si>
-  <si>
-    <t>MAJOR_GRD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GRADUATION_STATUS_DESCR, </t>
-  </si>
-  <si>
-    <t>represents year and month of matriculation term or start of bachelor's degree (your IR data may vary in this)</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>flag_transfer_credits_over_11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 or 0 </t>
-  </si>
-  <si>
-    <t>indicates if a student transferred with 12+ credit hours</t>
-  </si>
-  <si>
-    <t>flag_first_attempt</t>
-  </si>
-  <si>
-    <t>indicates if student record for course represents first attempt</t>
-  </si>
-  <si>
-    <t>years_before_course</t>
-  </si>
-  <si>
-    <t>demographics_high_school_GPA_standardized</t>
-  </si>
-  <si>
-    <t>difference in years from course_term and term_earliest</t>
-  </si>
-  <si>
-    <t>(demographics_high_school_GPA - demographics_high_school_GPA for cohort starting the same entry term) / demographics_high_school_GPA for cohort starting the same entry term</t>
-  </si>
-  <si>
-    <t>discipline_earliest_term</t>
-  </si>
-  <si>
-    <t>discipline_third_year_fall</t>
-  </si>
-  <si>
-    <t>bio_sci, phy_sci, eng_cs, other_STEM, non_STEM</t>
+    <t>level student graduated at</t>
+  </si>
+  <si>
+    <t>represents concentration associated with a specific term</t>
+  </si>
+  <si>
+    <t>concentration, abbreviated (e.g. EEO)</t>
+  </si>
+  <si>
+    <t>degree program level at term of graduation (BS, BA, etc)</t>
+  </si>
+  <si>
+    <t>concentration_term</t>
+  </si>
+  <si>
+    <t>CONCENTRATION</t>
+  </si>
+  <si>
+    <t>term_college</t>
+  </si>
+  <si>
+    <t>COLLEGE</t>
+  </si>
+  <si>
+    <t>DEGREE_LEVEL_GRADUATED</t>
   </si>
 </sst>
 </file>
@@ -1343,10 +1450,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table2" displayName="Table2" ref="A1:F49" totalsRowShown="0">
-  <autoFilter ref="A1:F49" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F44">
-    <sortCondition ref="A1:A44"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table2" displayName="Table2" ref="A1:F58" totalsRowShown="0">
+  <autoFilter ref="A1:F58" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F53">
+    <sortCondition ref="A1:A53"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="variable_name_project"/>
@@ -1677,15 +1784,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F49"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:F58"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="30.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="54.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="93.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="54.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="93.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1699,13 +1806,13 @@
         <v>72</v>
       </c>
       <c r="D1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
       </c>
       <c r="F1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -1838,21 +1945,21 @@
         <v>79</v>
       </c>
       <c r="F9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
+        <v>122</v>
+      </c>
+      <c r="D10" t="s">
         <v>123</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>124</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>125</v>
-      </c>
-      <c r="F10" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1874,10 +1981,10 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
+        <v>128</v>
+      </c>
+      <c r="B12" t="s">
         <v>129</v>
-      </c>
-      <c r="B12" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1961,10 +2068,10 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
+        <v>137</v>
+      </c>
+      <c r="B18" t="s">
         <v>138</v>
-      </c>
-      <c r="B18" t="s">
-        <v>139</v>
       </c>
       <c r="C18" t="s">
         <v>91</v>
@@ -1981,10 +2088,10 @@
         <v>38</v>
       </c>
       <c r="C19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1995,13 +2102,13 @@
         <v>44</v>
       </c>
       <c r="C20" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D20" t="s">
         <v>73</v>
       </c>
       <c r="E20" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2012,21 +2119,21 @@
         <v>40</v>
       </c>
       <c r="D21" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F21" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D22" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -2050,66 +2157,63 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>47</v>
+        <v>164</v>
       </c>
       <c r="B25" t="s">
-        <v>48</v>
+        <v>165</v>
+      </c>
+      <c r="D25" t="s">
+        <v>74</v>
+      </c>
+      <c r="E25" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>49</v>
+        <v>162</v>
       </c>
       <c r="B26" t="s">
-        <v>50</v>
-      </c>
-      <c r="C26" t="s">
-        <v>86</v>
+        <v>160</v>
       </c>
       <c r="D26" t="s">
         <v>74</v>
       </c>
       <c r="E26" t="s">
-        <v>127</v>
+        <v>163</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>9</v>
+        <v>47</v>
       </c>
       <c r="B27" t="s">
-        <v>10</v>
-      </c>
-      <c r="C27" t="s">
-        <v>94</v>
-      </c>
-      <c r="D27" t="s">
-        <v>93</v>
-      </c>
-      <c r="E27" t="s">
-        <v>95</v>
-      </c>
-      <c r="F27" t="s">
-        <v>119</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>15</v>
+        <v>49</v>
+      </c>
+      <c r="B28" t="s">
+        <v>50</v>
       </c>
       <c r="C28" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="D28" t="s">
-        <v>93</v>
-      </c>
-      <c r="F28" t="s">
-        <v>119</v>
+        <v>74</v>
+      </c>
+      <c r="E28" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" t="s">
-        <v>12</v>
+        <v>9</v>
+      </c>
+      <c r="B29" t="s">
+        <v>10</v>
       </c>
       <c r="C29" t="s">
         <v>94</v>
@@ -2118,18 +2222,15 @@
         <v>93</v>
       </c>
       <c r="E29" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F29" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" t="s">
-        <v>13</v>
-      </c>
-      <c r="B30" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C30" t="s">
         <v>94</v>
@@ -2137,16 +2238,13 @@
       <c r="D30" t="s">
         <v>93</v>
       </c>
-      <c r="E30" t="s">
-        <v>97</v>
-      </c>
       <c r="F30" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C31" t="s">
         <v>94</v>
@@ -2155,150 +2253,153 @@
         <v>93</v>
       </c>
       <c r="E31" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F31" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" t="s">
+        <v>159</v>
+      </c>
+      <c r="C32" t="s">
+        <v>94</v>
+      </c>
+      <c r="D32" t="s">
+        <v>93</v>
+      </c>
+      <c r="E32" t="s">
+        <v>161</v>
+      </c>
+      <c r="F32" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" t="s">
+        <v>13</v>
+      </c>
+      <c r="B33" t="s">
+        <v>14</v>
+      </c>
+      <c r="C33" t="s">
+        <v>94</v>
+      </c>
+      <c r="D33" t="s">
+        <v>93</v>
+      </c>
+      <c r="E33" t="s">
+        <v>97</v>
+      </c>
+      <c r="F33" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" t="s">
+        <v>11</v>
+      </c>
+      <c r="C34" t="s">
+        <v>94</v>
+      </c>
+      <c r="D34" t="s">
+        <v>93</v>
+      </c>
+      <c r="E34" t="s">
+        <v>98</v>
+      </c>
+      <c r="F34" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" t="s">
         <v>52</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B35" t="s">
+        <v>131</v>
+      </c>
+      <c r="D35" t="s">
         <v>132</v>
       </c>
-      <c r="D32" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5">
-      <c r="A33" t="s">
-        <v>136</v>
-      </c>
-      <c r="B33" t="s">
-        <v>148</v>
-      </c>
-      <c r="D33" t="s">
-        <v>73</v>
-      </c>
-      <c r="E33" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5">
-      <c r="A34" t="s">
-        <v>51</v>
-      </c>
-      <c r="C34" t="s">
-        <v>86</v>
-      </c>
-      <c r="D34" t="s">
-        <v>74</v>
-      </c>
-      <c r="E34" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5">
-      <c r="A35" t="s">
-        <v>144</v>
-      </c>
-      <c r="B35" t="s">
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" t="s">
+        <v>135</v>
+      </c>
+      <c r="B36" t="s">
         <v>145</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5">
-      <c r="A36" t="s">
-        <v>6</v>
-      </c>
-      <c r="B36" t="s">
-        <v>147</v>
-      </c>
-      <c r="C36" t="s">
-        <v>105</v>
       </c>
       <c r="D36" t="s">
         <v>73</v>
       </c>
       <c r="E36" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
       <c r="A37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B37" t="s">
-        <v>4</v>
+        <v>51</v>
       </c>
       <c r="C37" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="D37" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E37" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
       <c r="A38" t="s">
-        <v>5</v>
+        <v>180</v>
       </c>
       <c r="B38" t="s">
-        <v>146</v>
+        <v>190</v>
       </c>
       <c r="C38" t="s">
-        <v>105</v>
+        <v>182</v>
       </c>
       <c r="D38" t="s">
         <v>73</v>
       </c>
       <c r="E38" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
       <c r="A39" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B39" t="s">
-        <v>7</v>
-      </c>
-      <c r="C39" t="s">
-        <v>86</v>
-      </c>
-      <c r="D39" t="s">
-        <v>74</v>
-      </c>
-      <c r="E39" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
       <c r="A40" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B40" t="s">
-        <v>131</v>
+        <v>172</v>
       </c>
       <c r="C40" t="s">
-        <v>128</v>
+        <v>104</v>
       </c>
       <c r="D40" t="s">
-        <v>103</v>
+        <v>73</v>
       </c>
       <c r="E40" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
       <c r="A41" t="s">
-        <v>53</v>
+        <v>3</v>
       </c>
       <c r="B41" t="s">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="C41" t="s">
         <v>104</v>
@@ -2307,116 +2408,257 @@
         <v>73</v>
       </c>
       <c r="E41" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" t="s">
+        <v>5</v>
+      </c>
+      <c r="B42" t="s">
+        <v>167</v>
+      </c>
+      <c r="C42" t="s">
+        <v>104</v>
+      </c>
+      <c r="D42" t="s">
+        <v>73</v>
+      </c>
+      <c r="E42" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" t="s">
+        <v>173</v>
+      </c>
+      <c r="B43" t="s">
+        <v>174</v>
+      </c>
+      <c r="C43" t="s">
+        <v>175</v>
+      </c>
+      <c r="D43" t="s">
+        <v>73</v>
+      </c>
+      <c r="E43" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" t="s">
+        <v>186</v>
+      </c>
+      <c r="B44" t="s">
+        <v>187</v>
+      </c>
+      <c r="C44" t="s">
+        <v>184</v>
+      </c>
+      <c r="D44" t="s">
+        <v>73</v>
+      </c>
+      <c r="E44" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" t="s">
+        <v>134</v>
+      </c>
+      <c r="B45" t="s">
+        <v>7</v>
+      </c>
+      <c r="C45" t="s">
+        <v>86</v>
+      </c>
+      <c r="D45" t="s">
+        <v>74</v>
+      </c>
+      <c r="E45" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" t="s">
+        <v>8</v>
+      </c>
+      <c r="B46" t="s">
+        <v>130</v>
+      </c>
+      <c r="C46" t="s">
+        <v>127</v>
+      </c>
+      <c r="D46" t="s">
+        <v>103</v>
+      </c>
+      <c r="E46" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47" t="s">
+        <v>53</v>
+      </c>
+      <c r="B47" t="s">
+        <v>36</v>
+      </c>
+      <c r="C47" t="s">
+        <v>181</v>
+      </c>
+      <c r="D47" t="s">
+        <v>73</v>
+      </c>
+      <c r="E47" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
-      <c r="A42" t="s">
+    <row r="48" spans="1:6">
+      <c r="A48" t="s">
+        <v>139</v>
+      </c>
+      <c r="B48" t="s">
         <v>140</v>
       </c>
-      <c r="B42" t="s">
-        <v>141</v>
-      </c>
-      <c r="C42" t="s">
+      <c r="C48" t="s">
         <v>86</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D48" t="s">
         <v>74</v>
       </c>
-      <c r="E42" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5">
-      <c r="A43" t="s">
-        <v>143</v>
-      </c>
-      <c r="C43" t="s">
-        <v>66</v>
-      </c>
-      <c r="D43" t="s">
-        <v>74</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5">
-      <c r="A44" t="s">
-        <v>142</v>
-      </c>
-      <c r="B44" t="s">
-        <v>37</v>
-      </c>
-      <c r="C44" t="s">
-        <v>66</v>
-      </c>
-      <c r="D44" t="s">
-        <v>74</v>
-      </c>
-      <c r="E44" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5">
-      <c r="A45" t="s">
-        <v>151</v>
-      </c>
-      <c r="C45" t="s">
-        <v>152</v>
-      </c>
-      <c r="D45" t="s">
-        <v>93</v>
-      </c>
-      <c r="E45" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5">
-      <c r="A46" t="s">
-        <v>154</v>
-      </c>
-      <c r="C46" t="s">
-        <v>94</v>
-      </c>
-      <c r="D46" t="s">
-        <v>93</v>
-      </c>
-      <c r="E46" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5">
-      <c r="A47" t="s">
-        <v>156</v>
-      </c>
-      <c r="D47" t="s">
-        <v>124</v>
-      </c>
-      <c r="E47" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5">
-      <c r="A48" t="s">
-        <v>160</v>
-      </c>
-      <c r="D48" t="s">
-        <v>73</v>
-      </c>
       <c r="E48" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>161</v>
+        <v>168</v>
+      </c>
+      <c r="B49" t="s">
+        <v>169</v>
+      </c>
+      <c r="C49" t="s">
+        <v>86</v>
       </c>
       <c r="D49" t="s">
+        <v>74</v>
+      </c>
+      <c r="E49" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
+      <c r="A50" t="s">
+        <v>177</v>
+      </c>
+      <c r="B50" t="s">
+        <v>178</v>
+      </c>
+      <c r="D50" t="s">
         <v>73</v>
       </c>
-      <c r="E49" t="s">
-        <v>162</v>
+      <c r="E50" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5">
+      <c r="A51" t="s">
+        <v>188</v>
+      </c>
+      <c r="B51" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5">
+      <c r="A52" t="s">
+        <v>142</v>
+      </c>
+      <c r="C52" t="s">
+        <v>66</v>
+      </c>
+      <c r="D52" t="s">
+        <v>74</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
+      <c r="A53" t="s">
+        <v>141</v>
+      </c>
+      <c r="B53" t="s">
+        <v>37</v>
+      </c>
+      <c r="C53" t="s">
+        <v>66</v>
+      </c>
+      <c r="D53" t="s">
+        <v>74</v>
+      </c>
+      <c r="E53" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5">
+      <c r="A54" t="s">
+        <v>147</v>
+      </c>
+      <c r="C54" t="s">
+        <v>148</v>
+      </c>
+      <c r="D54" t="s">
+        <v>93</v>
+      </c>
+      <c r="E54" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
+      <c r="A55" t="s">
+        <v>150</v>
+      </c>
+      <c r="C55" t="s">
+        <v>94</v>
+      </c>
+      <c r="D55" t="s">
+        <v>93</v>
+      </c>
+      <c r="E55" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5">
+      <c r="A56" t="s">
+        <v>152</v>
+      </c>
+      <c r="D56" t="s">
+        <v>123</v>
+      </c>
+      <c r="E56" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57" t="s">
+        <v>156</v>
+      </c>
+      <c r="D57" t="s">
+        <v>73</v>
+      </c>
+      <c r="E57" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58" t="s">
+        <v>157</v>
+      </c>
+      <c r="D58" t="s">
+        <v>73</v>
+      </c>
+      <c r="E58" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -2431,36 +2673,36 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>